<commit_message>
hr: Wai Yan Aung 退職対応（2026-09-29）別紙 E1/E3/E4/E9/AWS特権ID を更新
Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/別紙/AWS特権ID利用記録_0205.xlsx
+++ b/別紙/AWS特権ID利用記録_0205.xlsx
@@ -32,12 +32,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D5F5E3"/>
+        <bgColor rgb="00D5F5E3"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -67,12 +73,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="20" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="標準" xfId="0" builtinId="0"/>
@@ -438,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q55"/>
+  <dimension ref="A1:Q56"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <cols>
     <col width="4" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -2356,6 +2363,66 @@
       <c r="P55" s="4" t="n"/>
       <c r="Q55" s="4" t="n"/>
     </row>
+    <row r="56">
+      <c r="A56" s="5" t="n">
+        <v>55</v>
+      </c>
+      <c r="B56" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>無効化</t>
+        </is>
+      </c>
+      <c r="D56" s="5" t="inlineStr">
+        <is>
+          <t>IAM</t>
+        </is>
+      </c>
+      <c r="E56" s="5" t="inlineStr">
+        <is>
+          <t>wii@codium.co</t>
+        </is>
+      </c>
+      <c r="F56" s="5" t="inlineStr">
+        <is>
+          <t>Wai Yan Aung</t>
+        </is>
+      </c>
+      <c r="G56" s="5" t="inlineStr">
+        <is>
+          <t>CODIUM</t>
+        </is>
+      </c>
+      <c r="H56" s="5" t="inlineStr">
+        <is>
+          <t>退職に伴うアカウント停止・アクセスキー削除</t>
+        </is>
+      </c>
+      <c r="I56" s="5" t="inlineStr">
+        <is>
+          <t>山田氏（Trello承認）</t>
+        </is>
+      </c>
+      <c r="J56" s="5" t="inlineStr">
+        <is>
+          <t>IAM Deactivate + アクセスキー削除 + MFA 削除</t>
+        </is>
+      </c>
+      <c r="K56" s="5" t="inlineStr">
+        <is>
+          <t>AWS IAM</t>
+        </is>
+      </c>
+      <c r="N56" s="5" t="inlineStr">
+        <is>
+          <t>無</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>